<commit_message>
Penamaan istilah standar SMK
</commit_message>
<xml_diff>
--- a/backend/uploads/Template_Import_Users.xlsx
+++ b/backend/uploads/Template_Import_Users.xlsx
@@ -398,15 +398,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="38.83203125" customWidth="1"/>
-    <col min="5" max="5" width="38.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="42.83203125" customWidth="1"/>
+    <col min="6" max="6" width="32.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -420,15 +421,18 @@
         <v>Role</v>
       </c>
       <c r="D1" t="str">
-        <v>Majority</v>
+        <v>Bidang Keahlian</v>
       </c>
       <c r="E1" t="str">
-        <v>StudyProgram</v>
+        <v>Program Keahlian</v>
       </c>
       <c r="F1" t="str">
+        <v>Konsentrasi Keahlian</v>
+      </c>
+      <c r="G1" t="str">
         <v>StudentId</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>NIP</v>
       </c>
     </row>
@@ -443,15 +447,18 @@
         <v>STUDENT</v>
       </c>
       <c r="D2" t="str">
-        <v>Teknik Komputer dan Jaringan</v>
+        <v>Teknologi Informasi</v>
       </c>
       <c r="E2" t="str">
-        <v>Teknik Komputer dan Informatika</v>
+        <v>Pengembangan Perangkat Lunak dan Gim</v>
       </c>
       <c r="F2" t="str">
+        <v>Rekayasa Perangkat Lunak</v>
+      </c>
+      <c r="G2" t="str">
         <v>20241001</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v/>
       </c>
     </row>
@@ -466,15 +473,18 @@
         <v>TEACHER</v>
       </c>
       <c r="D3" t="str">
-        <v>Teknik Komputer dan Jaringan</v>
+        <v>Teknologi Informasi</v>
       </c>
       <c r="E3" t="str">
-        <v>Teknik Komputer dan Informatika</v>
+        <v>Pengembangan Perangkat Lunak dan Gim</v>
       </c>
       <c r="F3" t="str">
+        <v>Rekayasa Perangkat Lunak</v>
+      </c>
+      <c r="G3" t="str">
         <v/>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>198501012010011001</v>
       </c>
     </row>
@@ -489,32 +499,35 @@
         <v>STUDENT</v>
       </c>
       <c r="D4" t="str">
-        <v>Pengembangan Perangkat Lunak dan Gim</v>
+        <v>Bisnis dan Manajemen</v>
       </c>
       <c r="E4" t="str">
-        <v>Rekayasa Perangkat Lunak</v>
+        <v>Akuntansi dan Keuangan Lembaga</v>
       </c>
       <c r="F4" t="str">
+        <v>Akuntansi</v>
+      </c>
+      <c r="G4" t="str">
         <v>20241002</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="65.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -522,10 +535,10 @@
         <v>Kolom</v>
       </c>
       <c r="B1" t="str">
-        <v>Wajib</v>
+        <v>Status</v>
       </c>
       <c r="C1" t="str">
-        <v>Keterangan</v>
+        <v>Penjelasan</v>
       </c>
     </row>
     <row r="2">
@@ -533,10 +546,10 @@
         <v>Name</v>
       </c>
       <c r="B2" t="str">
-        <v>Ya</v>
+        <v>Wajib</v>
       </c>
       <c r="C2" t="str">
-        <v>Nama lengkap user (siswa/guru)</v>
+        <v>Nama lengkap pengguna (siswa atau guru)</v>
       </c>
     </row>
     <row r="3">
@@ -544,10 +557,10 @@
         <v>Email</v>
       </c>
       <c r="B3" t="str">
-        <v>Ya</v>
+        <v>Wajib</v>
       </c>
       <c r="C3" t="str">
-        <v>Email aktif / unik untuk akun login</v>
+        <v>Email unik untuk akun login pengguna</v>
       </c>
     </row>
     <row r="4">
@@ -555,7 +568,7 @@
         <v>Role</v>
       </c>
       <c r="B4" t="str">
-        <v>Ya</v>
+        <v>Wajib</v>
       </c>
       <c r="C4" t="str">
         <v>Pilihan: STUDENT atau TEACHER</v>
@@ -563,51 +576,62 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Majority</v>
+        <v>Bidang Keahlian</v>
       </c>
       <c r="B5" t="str">
         <v>Opsional</v>
       </c>
       <c r="C5" t="str">
-        <v>Program / Konsentrasi Keahlian (misal: Rekayasa Perangkat Lunak)</v>
+        <v>Bidang Keahlian SMK (misal: Teknologi Informasi, Bisnis dan Manajemen)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>StudyProgram</v>
+        <v>Program Keahlian</v>
       </c>
       <c r="B6" t="str">
         <v>Opsional</v>
       </c>
       <c r="C6" t="str">
-        <v>Bidang / Program Studi Kejuruan</v>
+        <v>Program Keahlian SMK (misal: Pengembangan Perangkat Lunak dan Gim)</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>StudentId</v>
+        <v>Konsentrasi Keahlian</v>
       </c>
       <c r="B7" t="str">
-        <v>Siswa</v>
+        <v>Wajib</v>
       </c>
       <c r="C7" t="str">
-        <v>Nomor Induk Siswa / NIM / NISN (wajib jika Role STUDENT)</v>
+        <v>Konsentrasi Keahlian SMK (misal: Rekayasa Perangkat Lunak, Akuntansi)</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>StudentId</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Siswa</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Nomor Induk Siswa Nasional / NISN (wajib diisi untuk Role STUDENT)</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
         <v>NIP</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B9" t="str">
         <v>Guru</v>
       </c>
-      <c r="C8" t="str">
-        <v>Nomor Induk Pegawai (wajib jika Role TEACHER)</v>
+      <c r="C9" t="str">
+        <v>Nomor Induk Pegawai (wajib diisi untuk Role TEACHER)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>